<commit_message>
modified v3.1 data pipeline
</commit_message>
<xml_diff>
--- a/data/outputs/feature_dictionary.xlsx
+++ b/data/outputs/feature_dictionary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H175"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -966,7 +966,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Real Ookla test count where a real anchor exists for the cell; Poisson-simulated otherwise. Represents measurement VOLUME, not the outcome — safe as a feature in either target mode.</t>
+          <t>Simulated HOURLY-equivalent test count. For Ookla-anchored cells this is Poisson-sampled around an hourly rate derived from the REAL quarterly total (ookla_quarter_test_count / ~2160 hours, scaled by demand), NOT the quarterly total itself repeated per hour (that was a bug — see CHANGELOG). Represents measurement VOLUME, not the outcome — safe as a feature in either target mode.</t>
         </is>
       </c>
     </row>
@@ -1010,16 +1010,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>qoe_level_is_ookla_anchored</t>
+          <t>ookla_quarter_test_count</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>100</v>
+        <v>57.78</v>
       </c>
       <c r="E19" t="b">
         <v>1</v>
@@ -1030,7 +1030,7 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>True if a real Ookla quarterly average existed to re-centre this cell's simulated hourly values on (~41% of cells). False does not mean 'less real' shape — the hourly SHAPE is simulated either way.</t>
+          <t>REAL Ookla quarterly test count for this cell (constant across all 168 simulated hours by definition — it is a QUARTERLY total, never a per-hour figure). NaN if the cell has no Ookla tile coverage.</t>
         </is>
       </c>
     </row>
@@ -1042,27 +1042,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>qoe_hourly_shape_is_simulated</t>
+          <t>ookla_quarter_device_count</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>100</v>
+        <v>57.78</v>
       </c>
       <c r="E20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Always True. Included explicitly so this fact cannot be missed or confused with the anchored/unanchored distinction above. Excluded from ML features (constant, zero information).</t>
+          <t>REAL Ookla quarterly unique-device count for this cell (constant across all 168 simulated hours; quarterly, not hourly). NaN if unavailable in the source tile or no coverage exists.</t>
         </is>
       </c>
     </row>
@@ -1074,12 +1074,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>hour_of_day</t>
+          <t>qoe_baseline_source</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>int32</t>
+          <t>str</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1094,7 +1094,7 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
+          <t>Human-readable provenance string: 'ookla_q4_2024_static_anchor' or 'no_real_anchor_simulated_only'. Complements the qoe_level_is_ookla_anchored boolean.</t>
         </is>
       </c>
     </row>
@@ -1106,12 +1106,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>day_of_week</t>
+          <t>qoe_level_is_ookla_anchored</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>int32</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1126,7 +1126,7 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
+          <t>True if a real Ookla quarterly average existed to re-centre this cell's simulated hourly values on (~41% of cells). False does not mean 'less real' shape — the hourly SHAPE is simulated either way.</t>
         </is>
       </c>
     </row>
@@ -1138,27 +1138,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>is_weekend</t>
+          <t>qoe_hourly_shape_is_simulated</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D23" t="n">
         <v>100</v>
       </c>
       <c r="E23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
+          <t>Always True. Included explicitly so this fact cannot be missed or confused with the anchored/unanchored distinction above. Excluded from ML features (constant, zero information).</t>
         </is>
       </c>
     </row>
@@ -1170,12 +1170,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>is_peak_period</t>
+          <t>ridership_daily_surge_factor</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1190,7 +1190,7 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
+          <t>Real daily ridership-derived demand multiplier (normalized to the selected week's mean), summed only over Klang-Valley-relevant transit modes (national/inter-city services like ETS, Intercity, Komuter Utara, and Tebrau are excluded). Previously folded silently into the hourly formula with no standalone column; now exported directly so it can be inspected or used as its own feature.</t>
         </is>
       </c>
     </row>
@@ -1202,16 +1202,16 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>lag_1h_dl_median</t>
+          <t>hour_of_day</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int32</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="E25" t="b">
         <v>1</v>
@@ -1222,7 +1222,7 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Value of dl_median exactly 1 hour prior (shift(1), leakage-free).</t>
+          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
         </is>
       </c>
     </row>
@@ -1234,16 +1234,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>lag_2h_dl_median</t>
+          <t>day_of_week</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int32</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>98.81</v>
+        <v>100</v>
       </c>
       <c r="E26" t="b">
         <v>1</v>
@@ -1254,7 +1254,7 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Value of dl_median exactly 2 hours prior (shift(2), leakage-free).</t>
+          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
         </is>
       </c>
     </row>
@@ -1266,16 +1266,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>lag_24h_dl_median</t>
+          <t>is_weekend</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>85.70999999999999</v>
+        <v>100</v>
       </c>
       <c r="E27" t="b">
         <v>1</v>
@@ -1286,7 +1286,7 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Value of dl_median exactly 24 hours prior (shift(24), leakage-free).</t>
+          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
         </is>
       </c>
     </row>
@@ -1298,16 +1298,16 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>rolling_mean_24h_dl_median</t>
+          <t>is_peak_period</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="E28" t="b">
         <v>1</v>
@@ -1318,7 +1318,7 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Trailing rolling mean of 24h_dl_median, computed after shift(1) (leakage-free).</t>
+          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>rolling_std_24h_dl_median</t>
+          <t>lag_1h_dl_median</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>100</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E29" t="b">
         <v>1</v>
@@ -1350,7 +1350,7 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Trailing rolling standard deviation of 24h_dl_median, computed after shift(1) (leakage-free).</t>
+          <t>Value of dl_median exactly 1 hour prior (shift(1), leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1362,16 +1362,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>lag_1h_dl_median_valid</t>
+          <t>lag_2h_dl_median</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>100</v>
+        <v>98.81</v>
       </c>
       <c r="E30" t="b">
         <v>1</v>
@@ -1382,7 +1382,7 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Value of dl_median_valid exactly 1 hour prior (shift(1), leakage-free).</t>
+          <t>Value of dl_median exactly 2 hours prior (shift(2), leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1394,16 +1394,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>lag_2h_dl_median_valid</t>
+          <t>lag_24h_dl_median</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>100</v>
+        <v>85.70999999999999</v>
       </c>
       <c r="E31" t="b">
         <v>1</v>
@@ -1414,7 +1414,7 @@
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Value of dl_median_valid exactly 2 hours prior (shift(2), leakage-free).</t>
+          <t>Value of dl_median exactly 24 hours prior (shift(24), leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1426,16 +1426,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>lag_24h_dl_median_valid</t>
+          <t>rolling_mean_24h_dl_median</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>100</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E32" t="b">
         <v>1</v>
@@ -1446,7 +1446,7 @@
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Value of dl_median_valid exactly 24 hours prior (shift(24), leakage-free).</t>
+          <t>Trailing rolling mean of 24h_dl_median, computed after shift(1) (leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1458,12 +1458,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>rolling_mean_24h_dl_median_valid</t>
+          <t>rolling_std_24h_dl_median</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1478,7 +1478,7 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Trailing rolling mean of 24h_dl_median_valid, computed after shift(1) (leakage-free).</t>
+          <t>Trailing rolling standard deviation of 24h_dl_median, computed after shift(1) (leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1490,16 +1490,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>lag_1h_rtt_median</t>
+          <t>lag_1h_dl_median_valid</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="E34" t="b">
         <v>1</v>
@@ -1510,7 +1510,7 @@
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Value of rtt_median exactly 1 hour prior (shift(1), leakage-free).</t>
+          <t>Value of dl_median_valid exactly 1 hour prior (shift(1), leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1522,16 +1522,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>lag_2h_rtt_median</t>
+          <t>lag_2h_dl_median_valid</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>98.81</v>
+        <v>100</v>
       </c>
       <c r="E35" t="b">
         <v>1</v>
@@ -1542,7 +1542,7 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Value of rtt_median exactly 2 hours prior (shift(2), leakage-free).</t>
+          <t>Value of dl_median_valid exactly 2 hours prior (shift(2), leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1554,16 +1554,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>lag_24h_rtt_median</t>
+          <t>lag_24h_dl_median_valid</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>85.70999999999999</v>
+        <v>100</v>
       </c>
       <c r="E36" t="b">
         <v>1</v>
@@ -1574,7 +1574,7 @@
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Value of rtt_median exactly 24 hours prior (shift(24), leakage-free).</t>
+          <t>Value of dl_median_valid exactly 24 hours prior (shift(24), leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1586,16 +1586,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>rolling_mean_24h_rtt_median</t>
+          <t>rolling_mean_24h_dl_median_valid</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="E37" t="b">
         <v>1</v>
@@ -1606,7 +1606,7 @@
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Trailing rolling mean of 24h_rtt_median, computed after shift(1) (leakage-free).</t>
+          <t>Trailing rolling mean of 24h_dl_median_valid, computed after shift(1) (leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>rolling_std_24h_rtt_median</t>
+          <t>lag_1h_rtt_median</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>100</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E38" t="b">
         <v>1</v>
@@ -1638,7 +1638,7 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Trailing rolling standard deviation of 24h_rtt_median, computed after shift(1) (leakage-free).</t>
+          <t>Value of rtt_median exactly 1 hour prior (shift(1), leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1650,16 +1650,16 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>lag_1h_rtt_median_valid</t>
+          <t>lag_2h_rtt_median</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>100</v>
+        <v>98.81</v>
       </c>
       <c r="E39" t="b">
         <v>1</v>
@@ -1670,7 +1670,7 @@
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Value of rtt_median_valid exactly 1 hour prior (shift(1), leakage-free).</t>
+          <t>Value of rtt_median exactly 2 hours prior (shift(2), leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1682,16 +1682,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>lag_2h_rtt_median_valid</t>
+          <t>lag_24h_rtt_median</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>100</v>
+        <v>85.70999999999999</v>
       </c>
       <c r="E40" t="b">
         <v>1</v>
@@ -1702,7 +1702,7 @@
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Value of rtt_median_valid exactly 2 hours prior (shift(2), leakage-free).</t>
+          <t>Value of rtt_median exactly 24 hours prior (shift(24), leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1714,16 +1714,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>lag_24h_rtt_median_valid</t>
+          <t>rolling_mean_24h_rtt_median</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>100</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E41" t="b">
         <v>1</v>
@@ -1734,7 +1734,7 @@
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Value of rtt_median_valid exactly 24 hours prior (shift(24), leakage-free).</t>
+          <t>Trailing rolling mean of 24h_rtt_median, computed after shift(1) (leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1746,12 +1746,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>rolling_mean_24h_rtt_median_valid</t>
+          <t>rolling_std_24h_rtt_median</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1766,7 +1766,7 @@
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Trailing rolling mean of 24h_rtt_median_valid, computed after shift(1) (leakage-free).</t>
+          <t>Trailing rolling standard deviation of 24h_rtt_median, computed after shift(1) (leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1778,16 +1778,16 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>qoe_trend_1h</t>
+          <t>lag_1h_rtt_median_valid</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="E43" t="b">
         <v>1</v>
@@ -1798,7 +1798,7 @@
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
+          <t>Value of rtt_median_valid exactly 1 hour prior (shift(1), leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>in_warmup_window</t>
+          <t>lag_2h_rtt_median_valid</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1830,7 +1830,7 @@
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
+          <t>Value of rtt_median_valid exactly 2 hours prior (shift(2), leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>tower_count</t>
+          <t>lag_24h_rtt_median_valid</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1862,7 +1862,7 @@
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Deduplicated approximate PHYSICAL SITE count (OpenCellID records collapsed by ~11m coordinate rounding) — see opencellid_record_count for the raw, non-deduplicated record count.</t>
+          <t>Value of rtt_median_valid exactly 24 hours prior (shift(24), leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>opencellid_record_count</t>
+          <t>rolling_mean_24h_rtt_median_valid</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1894,7 +1894,7 @@
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Raw OpenCellID record count per cell BEFORE deduplication — includes multiple sectors/technologies/operators at the same physical site. Use tower_count for a physical-site estimate.</t>
+          <t>Trailing rolling mean of 24h_rtt_median_valid, computed after shift(1) (leakage-free).</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1906,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>tower_density_per_km2</t>
+          <t>qoe_trend_1h</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>100</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E47" t="b">
         <v>1</v>
@@ -1938,12 +1938,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>dist_to_nearest_tower_m</t>
+          <t>in_warmup_window</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1958,7 +1958,7 @@
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Real geometric nearest-neighbor distance (sjoin_nearest, projected CRS) from the cell centroid to the nearest deduplicated OpenCellID site.</t>
+          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
         </is>
       </c>
     </row>
@@ -1970,12 +1970,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>tower_is_synthetic</t>
+          <t>tower_count</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1990,7 +1990,7 @@
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>True if tower used a synthetic fallback (raw source file missing).</t>
+          <t>Deduplicated approximate PHYSICAL SITE count (OpenCellID records collapsed by ~11m coordinate rounding) — see opencellid_record_count for the raw, non-deduplicated record count.</t>
         </is>
       </c>
     </row>
@@ -2002,12 +2002,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>tower_source</t>
+          <t>opencellid_record_count</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2022,7 +2022,7 @@
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Provenance string: 'opencellid_deduplicated' (real) or 'synthetic_fallback_no_file'.</t>
+          <t>Raw OpenCellID record count per cell BEFORE deduplication — includes multiple sectors/technologies/operators at the same physical site. Use tower_count for a physical-site estimate.</t>
         </is>
       </c>
     </row>
@@ -2034,12 +2034,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>building_count</t>
+          <t>tower_density_per_km2</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2054,7 +2054,7 @@
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Real Google Open Buildings V3 footprint count per cell (confidence &gt;= 0.65 only).</t>
+          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>total_building_area_m2</t>
+          <t>dist_to_nearest_tower_m</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2086,7 +2086,7 @@
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Real summed footprint area (m^2) per cell.</t>
+          <t>Real geometric nearest-neighbor distance (sjoin_nearest, projected CRS) from the cell centroid to the nearest deduplicated OpenCellID site.</t>
         </is>
       </c>
     </row>
@@ -2098,12 +2098,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>built_up_ratio</t>
+          <t>tower_is_synthetic</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2118,7 +2118,7 @@
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Real building footprint area / real H3 cell area (both from GIS geometry, not a hardcoded constant).</t>
+          <t>True if tower used a synthetic fallback (raw source file missing).</t>
         </is>
       </c>
     </row>
@@ -2130,12 +2130,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>building_density_per_km2</t>
+          <t>tower_source</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -2150,7 +2150,7 @@
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>building_count / real cell area (km^2).</t>
+          <t>Provenance string: 'opencellid_deduplicated' (real) or 'synthetic_fallback_no_file'.</t>
         </is>
       </c>
     </row>
@@ -2162,12 +2162,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>avg_building_footprint_m2</t>
+          <t>building_count</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -2182,7 +2182,7 @@
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>total_building_area_m2 / building_count.</t>
+          <t>Real Google Open Buildings V3 footprint count per cell (confidence &gt;= 0.65 only).</t>
         </is>
       </c>
     </row>
@@ -2194,12 +2194,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>building_is_synthetic</t>
+          <t>total_building_area_m2</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -2214,7 +2214,7 @@
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
-          <t>True if building used a synthetic fallback (raw source file missing).</t>
+          <t>Real summed footprint area (m^2) per cell.</t>
         </is>
       </c>
     </row>
@@ -2226,12 +2226,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>poi_education_count</t>
+          <t>built_up_ratio</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -2246,7 +2246,7 @@
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Real OSM POI count: schools, universities, colleges, kindergartens.</t>
+          <t>Real building footprint area / real H3 cell area (both from GIS geometry, not a hardcoded constant).</t>
         </is>
       </c>
     </row>
@@ -2258,12 +2258,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>poi_healthcare_count</t>
+          <t>building_density_per_km2</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2278,7 +2278,7 @@
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Real OSM POI count: hospitals, clinics, pharmacies, doctors.</t>
+          <t>building_count / real cell area (km^2).</t>
         </is>
       </c>
     </row>
@@ -2290,12 +2290,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>poi_retail_food_count</t>
+          <t>avg_building_footprint_m2</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2310,7 +2310,7 @@
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Real OSM POI count: restaurants, cafes, fast food, shops.</t>
+          <t>total_building_area_m2 / building_count.</t>
         </is>
       </c>
     </row>
@@ -2322,12 +2322,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>poi_office_count</t>
+          <t>building_is_synthetic</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -2342,7 +2342,7 @@
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Real OSM POI count: tagged office=*.</t>
+          <t>True if building used a synthetic fallback (raw source file missing).</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>poi_recreation_count</t>
+          <t>poi_education_count</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2374,7 +2374,7 @@
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Real OSM POI count: leisure=* or tourism=*.</t>
+          <t>Real OSM POI count: schools, universities, colleges, kindergartens.</t>
         </is>
       </c>
     </row>
@@ -2386,12 +2386,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>road_length_m</t>
+          <t>poi_healthcare_count</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2406,7 +2406,7 @@
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Real road length (m) per cell via polygon overlay in a projected CRS (not a heuristic).</t>
+          <t>Real OSM POI count: hospitals, clinics, pharmacies, doctors.</t>
         </is>
       </c>
     </row>
@@ -2418,12 +2418,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>road_density_km_per_km2</t>
+          <t>poi_retail_food_count</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2438,7 +2438,7 @@
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>road_length_m / 1000 / real cell area (km^2).</t>
+          <t>Real OSM POI count: restaurants, cafes, fast food, shops.</t>
         </is>
       </c>
     </row>
@@ -2450,7 +2450,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>intersection_count</t>
+          <t>poi_office_count</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2470,7 +2470,7 @@
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Real OSM road-network node count per cell.</t>
+          <t>Real OSM POI count: tagged office=*.</t>
         </is>
       </c>
     </row>
@@ -2482,12 +2482,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>intersection_density_per_km2</t>
+          <t>poi_recreation_count</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -2502,7 +2502,7 @@
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>intersection_count / real cell area (km^2).</t>
+          <t>Real OSM POI count: leisure=* or tourism=*.</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>dist_to_nearest_transit_m</t>
+          <t>road_length_m</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2534,7 +2534,7 @@
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Real geometric nearest-neighbor distance to the nearest OSM transit/rail POI (sjoin_nearest, projected CRS).</t>
+          <t>Real road length (m) per cell via polygon overlay in a projected CRS (not a heuristic).</t>
         </is>
       </c>
     </row>
@@ -2546,12 +2546,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>poi_transport_stop_count</t>
+          <t>road_density_km_per_km2</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2566,7 +2566,7 @@
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Real OSM POI count of public-transport/rail stops joined into the cell.</t>
+          <t>road_length_m / 1000 / real cell area (km^2).</t>
         </is>
       </c>
     </row>
@@ -2578,12 +2578,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>osm_is_synthetic</t>
+          <t>intersection_count</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2598,7 +2598,7 @@
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
-          <t>True if osm used a synthetic fallback (raw source file missing).</t>
+          <t>Real OSM road-network node count per cell.</t>
         </is>
       </c>
     </row>
@@ -2610,7 +2610,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>population_night</t>
+          <t>intersection_density_per_km2</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2630,7 +2630,7 @@
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Real WorldPop 2020 zonal-statistics residential population estimate for the cell.</t>
+          <t>intersection_count / real cell area (km^2).</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>population_density_per_km2</t>
+          <t>dist_to_nearest_transit_m</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2662,7 +2662,7 @@
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>population_night / real cell area (km^2, projected CRS).</t>
+          <t>Real geometric nearest-neighbor distance to the nearest OSM transit/rail POI (sjoin_nearest, projected CRS).</t>
         </is>
       </c>
     </row>
@@ -2674,12 +2674,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>population_day</t>
+          <t>poi_transport_stop_count</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2694,7 +2694,7 @@
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Modelled daytime population (residential population reweighted by real OSM office/retail density) — explicitly an assumption, not a raster.</t>
+          <t>Real OSM POI count of public-transport/rail stops joined into the cell.</t>
         </is>
       </c>
     </row>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>population_is_synthetic</t>
+          <t>osm_is_synthetic</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2726,7 +2726,7 @@
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>True if population used a synthetic fallback (raw source file missing).</t>
+          <t>True if osm used a synthetic fallback (raw source file missing).</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>demand_pressure_base</t>
+          <t>population_night</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2758,7 +2758,7 @@
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t>0-100 composite of ONLY real static features (population, POI, built-up, roads/transport). Zero QoE dependency — safe to use with any target, any mode.</t>
+          <t>Real WorldPop 2020 zonal-statistics residential population estimate for the cell.</t>
         </is>
       </c>
     </row>
@@ -2770,7 +2770,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>demand_pressure_index_pre_spatial</t>
+          <t>population_density_per_km2</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2787,14 +2787,10 @@
       <c r="F74" t="b">
         <v>1</v>
       </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>Same circularity as demand_pressure_index, pre-spatial-smoothing.</t>
-        </is>
-      </c>
+      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>demand_pressure_base plus a historical-QoE component. Same circularity as demand_pressure_index, pre-spatial-smoothing.</t>
+          <t>population_night / real cell area (km^2, projected CRS).</t>
         </is>
       </c>
     </row>
@@ -2806,7 +2802,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>spatial_lag_dl_median</t>
+          <t>population_day</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2818,7 +2814,7 @@
         <v>100</v>
       </c>
       <c r="E75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F75" t="b">
         <v>1</v>
@@ -2826,7 +2822,7 @@
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Row-standardized H3 1-ring neighbor average of dl_median at the same timestamp (real libpysal weights).</t>
+          <t>Modelled daytime population (residential population reweighted by real OSM office/retail density) — explicitly an assumption, not a raster.</t>
         </is>
       </c>
     </row>
@@ -2838,12 +2834,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>spatial_var_dl_median</t>
+          <t>population_is_synthetic</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2858,7 +2854,7 @@
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Row-standardized H3 1-ring neighbor variance of dl_median at the same timestamp (real libpysal weights).</t>
+          <t>True if population used a synthetic fallback (raw source file missing).</t>
         </is>
       </c>
     </row>
@@ -2870,7 +2866,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>spatial_lag_rtt_median</t>
+          <t>demand_pressure_base</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2882,7 +2878,7 @@
         <v>100</v>
       </c>
       <c r="E77" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F77" t="b">
         <v>1</v>
@@ -2890,7 +2886,7 @@
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Row-standardized H3 1-ring neighbor average of rtt_median at the same timestamp (real libpysal weights).</t>
+          <t>0-100 composite of ONLY real static features (population, POI, built-up, roads/transport). Zero QoE dependency — safe to use with any target, any mode.</t>
         </is>
       </c>
     </row>
@@ -2902,7 +2898,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>spatial_var_rtt_median</t>
+          <t>demand_pressure_index_pre_spatial</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2919,10 +2915,14 @@
       <c r="F78" t="b">
         <v>1</v>
       </c>
-      <c r="G78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Same circularity as demand_pressure_index, pre-spatial-smoothing.</t>
+        </is>
+      </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Row-standardized H3 1-ring neighbor variance of rtt_median at the same timestamp (real libpysal weights).</t>
+          <t>demand_pressure_base plus a historical-QoE component. Same circularity as demand_pressure_index, pre-spatial-smoothing.</t>
         </is>
       </c>
     </row>
@@ -2934,7 +2934,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>spatial_lag_population_night</t>
+          <t>spatial_lag_dl_median</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2946,7 +2946,7 @@
         <v>100</v>
       </c>
       <c r="E79" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F79" t="b">
         <v>1</v>
@@ -2954,7 +2954,7 @@
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Row-standardized H3 1-ring neighbor average of population_night at the same timestamp (real libpysal weights).</t>
+          <t>Row-standardized H3 1-ring neighbor average of dl_median at the same timestamp (real libpysal weights).</t>
         </is>
       </c>
     </row>
@@ -2966,7 +2966,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>spatial_var_population_night</t>
+          <t>spatial_var_dl_median</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2986,7 +2986,7 @@
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Row-standardized H3 1-ring neighbor variance of population_night at the same timestamp (real libpysal weights).</t>
+          <t>Row-standardized H3 1-ring neighbor variance of dl_median at the same timestamp (real libpysal weights).</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>spatial_lag_demand_pressure_index_pre_spatial</t>
+          <t>spatial_lag_rtt_median</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3010,7 +3010,7 @@
         <v>100</v>
       </c>
       <c r="E81" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F81" t="b">
         <v>1</v>
@@ -3018,7 +3018,7 @@
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Row-standardized H3 1-ring neighbor average of demand_pressure_index_pre_spatial at the same timestamp (real libpysal weights).</t>
+          <t>Row-standardized H3 1-ring neighbor average of rtt_median at the same timestamp (real libpysal weights).</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>spatial_var_demand_pressure_index_pre_spatial</t>
+          <t>spatial_var_rtt_median</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3050,7 +3050,7 @@
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Row-standardized H3 1-ring neighbor variance of demand_pressure_index_pre_spatial at the same timestamp (real libpysal weights).</t>
+          <t>Row-standardized H3 1-ring neighbor variance of rtt_median at the same timestamp (real libpysal weights).</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>demand_pressure_index</t>
+          <t>spatial_lag_population_night</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3079,14 +3079,10 @@
       <c r="F83" t="b">
         <v>1</v>
       </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>Circular with the simulated QoE generator via its historical_qoe component (lag_24h_rtt_median). Use demand_pressure_base instead for a non-circular, real-data-only feature.</t>
-        </is>
-      </c>
+      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Final spatially-smoothed demand pressure index. Circular with the simulated QoE generator via its historical_qoe component (lag_24h_rtt_median). Use demand_pressure_base instead for a non-circular, real-data-only feature.</t>
+          <t>Row-standardized H3 1-ring neighbor average of population_night at the same timestamp (real libpysal weights).</t>
         </is>
       </c>
     </row>
@@ -3098,7 +3094,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>spatial_rolling_mean_24h_dl_median</t>
+          <t>spatial_var_population_night</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3118,7 +3114,7 @@
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
+          <t>Row-standardized H3 1-ring neighbor variance of population_night at the same timestamp (real libpysal weights).</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3126,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>gi_star_zscore_rtt_median</t>
+          <t>spatial_lag_demand_pressure_index_pre_spatial</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3150,7 +3146,7 @@
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Real Getis-Ord Gi* z-score for latency (esda.G_Local, star=True) — the full Gi* expectation/variance formulation, not a plain standardized neighbor average.</t>
+          <t>Row-standardized H3 1-ring neighbor average of demand_pressure_index_pre_spatial at the same timestamp (real libpysal weights).</t>
         </is>
       </c>
     </row>
@@ -3162,12 +3158,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>gi_star_pvalue_rtt_median</t>
+          <t>spatial_var_demand_pressure_index_pre_spatial</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>float32</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3182,7 +3178,7 @@
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Permutation-based p-value (99 permutations) for the Getis-Ord Gi* statistic on rtt_median.</t>
+          <t>Row-standardized H3 1-ring neighbor variance of demand_pressure_index_pre_spatial at the same timestamp (real libpysal weights).</t>
         </is>
       </c>
     </row>
@@ -3194,12 +3190,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>hotspot_category_rtt_median</t>
+          <t>demand_pressure_index</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -3211,10 +3207,14 @@
       <c r="F87" t="b">
         <v>1</v>
       </c>
-      <c r="G87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Circular with the simulated QoE generator via its historical_qoe component (lag_24h_rtt_median). Use demand_pressure_base instead for a non-circular, real-data-only feature.</t>
+        </is>
+      </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Hot/cold spot classification at 90/95/99% confidence, from real esda.G_Local p-values.</t>
+          <t>Final spatially-smoothed demand pressure index. Circular with the simulated QoE generator via its historical_qoe component (lag_24h_rtt_median). Use demand_pressure_base instead for a non-circular, real-data-only feature.</t>
         </is>
       </c>
     </row>
@@ -3226,7 +3226,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>local_moran_i_rtt_median</t>
+          <t>spatial_rolling_mean_24h_dl_median</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3246,7 +3246,7 @@
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Local Moran's I statistic value for rtt_median (real esda.Moran_Local).</t>
+          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3258,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>local_moran_pvalue_rtt_median</t>
+          <t>gi_star_zscore_rtt_median</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3278,7 +3278,7 @@
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Permutation-based p-value (99 permutations) for Local Moran's I on rtt_median.</t>
+          <t>Real Getis-Ord Gi* z-score for latency (esda.G_Local, star=True) — the full Gi* expectation/variance formulation, not a plain standardized neighbor average.</t>
         </is>
       </c>
     </row>
@@ -3290,12 +3290,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>local_moran_quadrant_rtt_median</t>
+          <t>gi_star_pvalue_rtt_median</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float32</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -3310,7 +3310,7 @@
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>HH/LH/LL/HL spatial cluster/outlier classification (real esda.Moran_Local).</t>
+          <t>Permutation-based p-value (99 permutations) for the Getis-Ord Gi* statistic on rtt_median.</t>
         </is>
       </c>
     </row>
@@ -3322,27 +3322,27 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>historical_hotspot_freq_rtt_median</t>
+          <t>hotspot_category_rtt_median</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="D91" t="n">
         <v>100</v>
       </c>
       <c r="E91" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F91" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Rolling (shift(1)-based, leakage-free) fraction of past hours this cell was a real (esda-confirmed) hotspot.</t>
+          <t>Hot/cold spot classification at 90/95/99% confidence, from real esda.G_Local p-values.</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>target_qoe_index</t>
+          <t>local_moran_i_rtt_median</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3366,15 +3366,15 @@
         <v>100</v>
       </c>
       <c r="E92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Custom composite 0-100 QoE index (log-utility download/upload minus exponential latency/loss penalty). NOT a validated ITU-T G.107 MOS — see qoe_target.py docstring.</t>
+          <t>Local Moran's I statistic value for rtt_median (real esda.Moran_Local).</t>
         </is>
       </c>
     </row>
@@ -3386,7 +3386,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>target_service_quality_1to5</t>
+          <t>local_moran_pvalue_rtt_median</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -3398,15 +3398,15 @@
         <v>100</v>
       </c>
       <c r="E93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1-5 linear rescaling of target_qoe_index. NOT a validated MOS/ACR score.</t>
+          <t>Permutation-based p-value (99 permutations) for Local Moran's I on rtt_median.</t>
         </is>
       </c>
     </row>
@@ -3418,12 +3418,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>target_is_degraded</t>
+          <t>local_moran_quadrant_rtt_median</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -3438,7 +3438,7 @@
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Binary SAME-HOUR degradation flag, derived from target_degradation_class &gt;= 1 (single shared threshold source — config.QOE_THRESHOLDS — so this can no longer disagree with target_degradation_class).</t>
+          <t>HH/LH/LL/HL spatial cluster/outlier classification (real esda.Moran_Local).</t>
         </is>
       </c>
     </row>
@@ -3450,27 +3450,27 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>target_degradation_class</t>
+          <t>historical_hotspot_freq_rtt_median</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D95" t="n">
         <v>100</v>
       </c>
       <c r="E95" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F95" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>0=normal, 1=degraded, 2=severe. Same threshold source as target_is_degraded.</t>
+          <t>Rolling (shift(1)-based, leakage-free) fraction of past hours this cell was a real (esda-confirmed) hotspot.</t>
         </is>
       </c>
     </row>
@@ -3482,12 +3482,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>qoe_confidence_score</t>
+          <t>hotspot_category_rtt_median_encoded</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -3502,7 +3502,7 @@
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
-          <t>min(1.0, test_sample_count / 10) — higher sample count = more confidence in the cell-hour's QoE estimate.</t>
+          <t>Ordinal-encoded hotspot confidence band (0=cold_99, 1=cold_95, 2=cold_90, 3=not_significant, 4=hot_90, 5=hot_95, 6=hot_99). ML-compatible integer version of hotspot_category_rtt_median (string, kept for dashboard).</t>
         </is>
       </c>
     </row>
@@ -3514,27 +3514,27 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>target_is_degraded_next_1h</t>
+          <t>local_moran_quadrant_rtt_median_encoded</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="E97" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F97" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
-          <t>RECOMMENDED PRIMARY ML TARGET. target_is_degraded shifted -1 per cell (groupby h3_index).shift(-1) — genuinely predicting the future, not classifying the present. NaN/0-valid for each cell's final row (no future observation exists).</t>
+          <t>Ordinal-encoded Local Moran's I spatial cluster/outlier class (0=not_significant, 1=LL, 2=LH, 3=HL, 4=HH). ML-compatible integer version of local_moran_quadrant_rtt_median (string, kept for dashboard).</t>
         </is>
       </c>
     </row>
@@ -3546,7 +3546,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>target_degradation_class_next_1h</t>
+          <t>target_qoe_index</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="E98" t="b">
         <v>0</v>
@@ -3566,7 +3566,7 @@
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
-          <t>3-class version of the next-hour forecast target.</t>
+          <t>Custom composite 0-100 QoE index (log-utility download/upload minus exponential latency/loss penalty). NOT a validated ITU-T G.107 MOS — see qoe_target.py docstring.</t>
         </is>
       </c>
     </row>
@@ -3578,7 +3578,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>target_qoe_index_next_1h</t>
+          <t>target_service_quality_1to5</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="E99" t="b">
         <v>0</v>
@@ -3598,7 +3598,7 @@
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Continuous version of the next-hour forecast target.</t>
+          <t>1-5 linear rescaling of target_qoe_index. NOT a validated MOS/ACR score.</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3610,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>target_next_1h_valid</t>
+          <t>target_is_degraded</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3630,56 +3630,56 @@
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1 if a real future observation existed to build the next-hour target from; 0 for each cell's final row. Drop rows where this is 0 before training — do not treat them as a 'not degraded' case.</t>
+          <t>Binary SAME-HOUR degradation flag, derived from target_degradation_class &gt;= 1 (single shared threshold source — config.QOE_THRESHOLDS — so this can no longer disagree with target_degradation_class).</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>cell_static_features</t>
+          <t>cell_time_dataset</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>h3_index</t>
+          <t>target_degradation_class</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D101" t="n">
         <v>100</v>
       </c>
       <c r="E101" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F101" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Uber H3 res-8 cell identifier (join key).</t>
+          <t>0=normal, 1=degraded, 2=severe. Same threshold source as target_is_degraded.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>cell_static_features</t>
+          <t>cell_time_dataset</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>tower_count</t>
+          <t>qoe_confidence_score</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3694,51 +3694,51 @@
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
         <is>
-          <t>Deduplicated approximate PHYSICAL SITE count (OpenCellID records collapsed by ~11m coordinate rounding) — see opencellid_record_count for the raw, non-deduplicated record count.</t>
+          <t>min(1.0, test_sample_count / 10) — higher sample count = more confidence in the cell-hour's QoE estimate.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>cell_static_features</t>
+          <t>cell_time_dataset</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>opencellid_record_count</t>
+          <t>target_is_degraded_next_1h</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>100</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E103" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F103" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Raw OpenCellID record count per cell BEFORE deduplication — includes multiple sectors/technologies/operators at the same physical site. Use tower_count for a physical-site estimate.</t>
+          <t>RECOMMENDED PRIMARY ML TARGET. target_is_degraded shifted -1 per cell (groupby h3_index).shift(-1) — genuinely predicting the future, not classifying the present. NaN/0-valid for each cell's final row (no future observation exists).</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>cell_static_features</t>
+          <t>cell_time_dataset</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>tower_density_per_km2</t>
+          <t>target_degradation_class_next_1h</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -3747,30 +3747,30 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>100</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E104" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F104" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
+          <t>3-class version of the next-hour forecast target.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>cell_static_features</t>
+          <t>cell_time_dataset</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>dist_to_nearest_tower_m</t>
+          <t>target_qoe_index_next_1h</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -3779,114 +3779,114 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>100</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E105" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F105" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Real geometric nearest-neighbor distance (sjoin_nearest, projected CRS) from the cell centroid to the nearest deduplicated OpenCellID site.</t>
+          <t>Continuous version of the next-hour forecast target.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>cell_static_features</t>
+          <t>cell_time_dataset</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>tower_is_synthetic</t>
+          <t>target_next_1h_valid</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D106" t="n">
         <v>100</v>
       </c>
       <c r="E106" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F106" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
-          <t>True if tower used a synthetic fallback (raw source file missing).</t>
+          <t>1 if a real future observation existed to build the next-hour target from; 0 for each cell's final row. Drop rows where this is 0 before training — do not treat them as a 'not degraded' case.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>cell_static_features</t>
+          <t>cell_time_dataset</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>tower_source</t>
+          <t>priority_exposure_score</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D107" t="n">
         <v>100</v>
       </c>
       <c r="E107" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F107" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Provenance string: 'opencellid_deduplicated' (real) or 'synthetic_fallback_no_file'.</t>
+          <t>MinMax-scaled population_day floored at 0.01 — the population-exposure component of the Priority Score. Not an ML feature (derived from population_day).</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>cell_static_features</t>
+          <t>cell_time_dataset</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>building_count</t>
+          <t>priority_base_score</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D108" t="n">
         <v>100</v>
       </c>
       <c r="E108" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F108" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
-          <t>Real Google Open Buildings V3 footprint count per cell (confidence &gt;= 0.65 only).</t>
+          <t>priority_exposure_score × historical_hotspot_freq × max(0.1, qoe_confidence_score) — pre-computed Priority Score base without model risk probability. Dashboard: final_priority = model_predicted_risk × priority_base_score. Not an ML feature.</t>
         </is>
       </c>
     </row>
@@ -3898,12 +3898,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>total_building_area_m2</t>
+          <t>h3_index</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3918,7 +3918,7 @@
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr">
         <is>
-          <t>Real summed footprint area (m^2) per cell.</t>
+          <t>Uber H3 res-8 cell identifier (join key).</t>
         </is>
       </c>
     </row>
@@ -3930,12 +3930,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>built_up_ratio</t>
+          <t>tower_count</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3950,7 +3950,7 @@
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Real building footprint area / real H3 cell area (both from GIS geometry, not a hardcoded constant).</t>
+          <t>Deduplicated approximate PHYSICAL SITE count (OpenCellID records collapsed by ~11m coordinate rounding) — see opencellid_record_count for the raw, non-deduplicated record count.</t>
         </is>
       </c>
     </row>
@@ -3962,12 +3962,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>building_density_per_km2</t>
+          <t>opencellid_record_count</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3982,7 +3982,7 @@
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr">
         <is>
-          <t>building_count / real cell area (km^2).</t>
+          <t>Raw OpenCellID record count per cell BEFORE deduplication — includes multiple sectors/technologies/operators at the same physical site. Use tower_count for a physical-site estimate.</t>
         </is>
       </c>
     </row>
@@ -3994,7 +3994,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>avg_building_footprint_m2</t>
+          <t>tower_density_per_km2</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -4014,7 +4014,7 @@
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
-          <t>total_building_area_m2 / building_count.</t>
+          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
         </is>
       </c>
     </row>
@@ -4026,12 +4026,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>building_is_synthetic</t>
+          <t>dist_to_nearest_tower_m</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -4046,7 +4046,7 @@
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr">
         <is>
-          <t>True if building used a synthetic fallback (raw source file missing).</t>
+          <t>Real geometric nearest-neighbor distance (sjoin_nearest, projected CRS) from the cell centroid to the nearest deduplicated OpenCellID site.</t>
         </is>
       </c>
     </row>
@@ -4058,12 +4058,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>poi_education_count</t>
+          <t>tower_is_synthetic</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -4078,7 +4078,7 @@
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr">
         <is>
-          <t>Real OSM POI count: schools, universities, colleges, kindergartens.</t>
+          <t>True if tower used a synthetic fallback (raw source file missing).</t>
         </is>
       </c>
     </row>
@@ -4090,12 +4090,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>poi_healthcare_count</t>
+          <t>tower_source</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -4110,7 +4110,7 @@
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Real OSM POI count: hospitals, clinics, pharmacies, doctors.</t>
+          <t>Provenance string: 'opencellid_deduplicated' (real) or 'synthetic_fallback_no_file'.</t>
         </is>
       </c>
     </row>
@@ -4122,7 +4122,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>poi_retail_food_count</t>
+          <t>building_count</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -4142,7 +4142,7 @@
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Real OSM POI count: restaurants, cafes, fast food, shops.</t>
+          <t>Real Google Open Buildings V3 footprint count per cell (confidence &gt;= 0.65 only).</t>
         </is>
       </c>
     </row>
@@ -4154,12 +4154,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>poi_office_count</t>
+          <t>total_building_area_m2</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -4174,7 +4174,7 @@
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Real OSM POI count: tagged office=*.</t>
+          <t>Real summed footprint area (m^2) per cell.</t>
         </is>
       </c>
     </row>
@@ -4186,12 +4186,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>poi_recreation_count</t>
+          <t>built_up_ratio</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -4206,7 +4206,7 @@
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Real OSM POI count: leisure=* or tourism=*.</t>
+          <t>Real building footprint area / real H3 cell area (both from GIS geometry, not a hardcoded constant).</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4218,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>road_length_m</t>
+          <t>building_density_per_km2</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -4238,7 +4238,7 @@
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr">
         <is>
-          <t>Real road length (m) per cell via polygon overlay in a projected CRS (not a heuristic).</t>
+          <t>building_count / real cell area (km^2).</t>
         </is>
       </c>
     </row>
@@ -4250,7 +4250,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>road_density_km_per_km2</t>
+          <t>avg_building_footprint_m2</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -4270,7 +4270,7 @@
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr">
         <is>
-          <t>road_length_m / 1000 / real cell area (km^2).</t>
+          <t>total_building_area_m2 / building_count.</t>
         </is>
       </c>
     </row>
@@ -4282,12 +4282,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>intersection_count</t>
+          <t>building_is_synthetic</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -4302,7 +4302,7 @@
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Real OSM road-network node count per cell.</t>
+          <t>True if building used a synthetic fallback (raw source file missing).</t>
         </is>
       </c>
     </row>
@@ -4314,12 +4314,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>intersection_density_per_km2</t>
+          <t>poi_education_count</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -4334,7 +4334,7 @@
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr">
         <is>
-          <t>intersection_count / real cell area (km^2).</t>
+          <t>Real OSM POI count: schools, universities, colleges, kindergartens.</t>
         </is>
       </c>
     </row>
@@ -4346,12 +4346,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>dist_to_nearest_transit_m</t>
+          <t>poi_healthcare_count</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -4366,7 +4366,7 @@
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr">
         <is>
-          <t>Real geometric nearest-neighbor distance to the nearest OSM transit/rail POI (sjoin_nearest, projected CRS).</t>
+          <t>Real OSM POI count: hospitals, clinics, pharmacies, doctors.</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>poi_transport_stop_count</t>
+          <t>poi_retail_food_count</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -4398,7 +4398,7 @@
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr">
         <is>
-          <t>Real OSM POI count of public-transport/rail stops joined into the cell.</t>
+          <t>Real OSM POI count: restaurants, cafes, fast food, shops.</t>
         </is>
       </c>
     </row>
@@ -4410,12 +4410,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>osm_is_synthetic</t>
+          <t>poi_office_count</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -4430,7 +4430,7 @@
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr">
         <is>
-          <t>True if osm used a synthetic fallback (raw source file missing).</t>
+          <t>Real OSM POI count: tagged office=*.</t>
         </is>
       </c>
     </row>
@@ -4442,12 +4442,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>population_night</t>
+          <t>poi_recreation_count</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -4462,7 +4462,7 @@
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Real WorldPop 2020 zonal-statistics residential population estimate for the cell.</t>
+          <t>Real OSM POI count: leisure=* or tourism=*.</t>
         </is>
       </c>
     </row>
@@ -4474,7 +4474,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>population_density_per_km2</t>
+          <t>road_length_m</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -4494,7 +4494,7 @@
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr">
         <is>
-          <t>population_night / real cell area (km^2, projected CRS).</t>
+          <t>Real road length (m) per cell via polygon overlay in a projected CRS (not a heuristic).</t>
         </is>
       </c>
     </row>
@@ -4506,7 +4506,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>population_day</t>
+          <t>road_density_km_per_km2</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -4526,7 +4526,7 @@
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
-          <t>Modelled daytime population (residential population reweighted by real OSM office/retail density) — explicitly an assumption, not a raster.</t>
+          <t>road_length_m / 1000 / real cell area (km^2).</t>
         </is>
       </c>
     </row>
@@ -4538,12 +4538,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>population_is_synthetic</t>
+          <t>intersection_count</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -4558,24 +4558,24 @@
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr">
         <is>
-          <t>True if population used a synthetic fallback (raw source file missing).</t>
+          <t>Real OSM road-network node count per cell.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>cell_static_qoe_baseline</t>
+          <t>cell_static_features</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>h3_index</t>
+          <t>intersection_density_per_km2</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -4590,24 +4590,24 @@
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr">
         <is>
-          <t>Uber H3 res-8 cell identifier (join key).</t>
+          <t>intersection_count / real cell area (km^2).</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>cell_static_qoe_baseline</t>
+          <t>cell_static_features</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>tower_count</t>
+          <t>dist_to_nearest_transit_m</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -4622,19 +4622,19 @@
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr">
         <is>
-          <t>Deduplicated approximate PHYSICAL SITE count (OpenCellID records collapsed by ~11m coordinate rounding) — see opencellid_record_count for the raw, non-deduplicated record count.</t>
+          <t>Real geometric nearest-neighbor distance to the nearest OSM transit/rail POI (sjoin_nearest, projected CRS).</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>cell_static_qoe_baseline</t>
+          <t>cell_static_features</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>opencellid_record_count</t>
+          <t>poi_transport_stop_count</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -4654,24 +4654,24 @@
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr">
         <is>
-          <t>Raw OpenCellID record count per cell BEFORE deduplication — includes multiple sectors/technologies/operators at the same physical site. Use tower_count for a physical-site estimate.</t>
+          <t>Real OSM POI count of public-transport/rail stops joined into the cell.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>cell_static_qoe_baseline</t>
+          <t>cell_static_features</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>tower_density_per_km2</t>
+          <t>osm_is_synthetic</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -4686,19 +4686,19 @@
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr">
         <is>
-          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
+          <t>True if osm used a synthetic fallback (raw source file missing).</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>cell_static_qoe_baseline</t>
+          <t>cell_static_features</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>dist_to_nearest_tower_m</t>
+          <t>population_night</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -4718,24 +4718,24 @@
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr">
         <is>
-          <t>Real geometric nearest-neighbor distance (sjoin_nearest, projected CRS) from the cell centroid to the nearest deduplicated OpenCellID site.</t>
+          <t>Real WorldPop 2020 zonal-statistics residential population estimate for the cell.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>cell_static_qoe_baseline</t>
+          <t>cell_static_features</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>tower_is_synthetic</t>
+          <t>population_density_per_km2</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -4750,24 +4750,24 @@
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr">
         <is>
-          <t>True if tower used a synthetic fallback (raw source file missing).</t>
+          <t>population_night / real cell area (km^2, projected CRS).</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>cell_static_qoe_baseline</t>
+          <t>cell_static_features</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>tower_source</t>
+          <t>population_day</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -4782,24 +4782,24 @@
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Provenance string: 'opencellid_deduplicated' (real) or 'synthetic_fallback_no_file'.</t>
+          <t>Modelled daytime population (residential population reweighted by real OSM office/retail density) — explicitly an assumption, not a raster.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>cell_static_qoe_baseline</t>
+          <t>cell_static_features</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>building_count</t>
+          <t>population_is_synthetic</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4814,19 +4814,19 @@
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Real Google Open Buildings V3 footprint count per cell (confidence &gt;= 0.65 only).</t>
+          <t>True if population used a synthetic fallback (raw source file missing).</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>cell_static_qoe_baseline</t>
+          <t>cell_static_features</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>total_building_area_m2</t>
+          <t>demand_pressure_base</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -4846,7 +4846,7 @@
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr">
         <is>
-          <t>Real summed footprint area (m^2) per cell.</t>
+          <t>0-100 composite of ONLY real static features (population, POI, built-up, roads/transport). Zero QoE dependency — safe to use with any target, any mode.</t>
         </is>
       </c>
     </row>
@@ -4858,12 +4858,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>built_up_ratio</t>
+          <t>h3_index</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -4878,7 +4878,7 @@
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr">
         <is>
-          <t>Real building footprint area / real H3 cell area (both from GIS geometry, not a hardcoded constant).</t>
+          <t>Uber H3 res-8 cell identifier (join key).</t>
         </is>
       </c>
     </row>
@@ -4890,12 +4890,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>building_density_per_km2</t>
+          <t>tower_count</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4910,7 +4910,7 @@
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr">
         <is>
-          <t>building_count / real cell area (km^2).</t>
+          <t>Deduplicated approximate PHYSICAL SITE count (OpenCellID records collapsed by ~11m coordinate rounding) — see opencellid_record_count for the raw, non-deduplicated record count.</t>
         </is>
       </c>
     </row>
@@ -4922,12 +4922,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>avg_building_footprint_m2</t>
+          <t>opencellid_record_count</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -4942,7 +4942,7 @@
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr">
         <is>
-          <t>total_building_area_m2 / building_count.</t>
+          <t>Raw OpenCellID record count per cell BEFORE deduplication — includes multiple sectors/technologies/operators at the same physical site. Use tower_count for a physical-site estimate.</t>
         </is>
       </c>
     </row>
@@ -4954,12 +4954,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>building_is_synthetic</t>
+          <t>tower_density_per_km2</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -4974,7 +4974,7 @@
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr">
         <is>
-          <t>True if building used a synthetic fallback (raw source file missing).</t>
+          <t>Undocumented — flag for the Data/GIS lead rather than guessing; do not assume this column is safe to use as-is.</t>
         </is>
       </c>
     </row>
@@ -4986,12 +4986,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>poi_education_count</t>
+          <t>dist_to_nearest_tower_m</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -5006,7 +5006,7 @@
       <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr">
         <is>
-          <t>Real OSM POI count: schools, universities, colleges, kindergartens.</t>
+          <t>Real geometric nearest-neighbor distance (sjoin_nearest, projected CRS) from the cell centroid to the nearest deduplicated OpenCellID site.</t>
         </is>
       </c>
     </row>
@@ -5018,12 +5018,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>poi_healthcare_count</t>
+          <t>tower_is_synthetic</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -5038,7 +5038,7 @@
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr">
         <is>
-          <t>Real OSM POI count: hospitals, clinics, pharmacies, doctors.</t>
+          <t>True if tower used a synthetic fallback (raw source file missing).</t>
         </is>
       </c>
     </row>
@@ -5050,12 +5050,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>poi_retail_food_count</t>
+          <t>tower_source</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -5070,7 +5070,7 @@
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr">
         <is>
-          <t>Real OSM POI count: restaurants, cafes, fast food, shops.</t>
+          <t>Provenance string: 'opencellid_deduplicated' (real) or 'synthetic_fallback_no_file'.</t>
         </is>
       </c>
     </row>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>poi_office_count</t>
+          <t>building_count</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -5102,7 +5102,7 @@
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr">
         <is>
-          <t>Real OSM POI count: tagged office=*.</t>
+          <t>Real Google Open Buildings V3 footprint count per cell (confidence &gt;= 0.65 only).</t>
         </is>
       </c>
     </row>
@@ -5114,12 +5114,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>poi_recreation_count</t>
+          <t>total_building_area_m2</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -5134,7 +5134,7 @@
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr">
         <is>
-          <t>Real OSM POI count: leisure=* or tourism=*.</t>
+          <t>Real summed footprint area (m^2) per cell.</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>road_length_m</t>
+          <t>built_up_ratio</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -5166,7 +5166,7 @@
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
-          <t>Real road length (m) per cell via polygon overlay in a projected CRS (not a heuristic).</t>
+          <t>Real building footprint area / real H3 cell area (both from GIS geometry, not a hardcoded constant).</t>
         </is>
       </c>
     </row>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>road_density_km_per_km2</t>
+          <t>building_density_per_km2</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -5198,7 +5198,7 @@
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
-          <t>road_length_m / 1000 / real cell area (km^2).</t>
+          <t>building_count / real cell area (km^2).</t>
         </is>
       </c>
     </row>
@@ -5210,12 +5210,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>intersection_count</t>
+          <t>avg_building_footprint_m2</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -5230,7 +5230,7 @@
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr">
         <is>
-          <t>Real OSM road-network node count per cell.</t>
+          <t>total_building_area_m2 / building_count.</t>
         </is>
       </c>
     </row>
@@ -5242,12 +5242,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>intersection_density_per_km2</t>
+          <t>building_is_synthetic</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -5262,7 +5262,7 @@
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr">
         <is>
-          <t>intersection_count / real cell area (km^2).</t>
+          <t>True if building used a synthetic fallback (raw source file missing).</t>
         </is>
       </c>
     </row>
@@ -5274,12 +5274,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>dist_to_nearest_transit_m</t>
+          <t>poi_education_count</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -5294,7 +5294,7 @@
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr">
         <is>
-          <t>Real geometric nearest-neighbor distance to the nearest OSM transit/rail POI (sjoin_nearest, projected CRS).</t>
+          <t>Real OSM POI count: schools, universities, colleges, kindergartens.</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>poi_transport_stop_count</t>
+          <t>poi_healthcare_count</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -5326,7 +5326,7 @@
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr">
         <is>
-          <t>Real OSM POI count of public-transport/rail stops joined into the cell.</t>
+          <t>Real OSM POI count: hospitals, clinics, pharmacies, doctors.</t>
         </is>
       </c>
     </row>
@@ -5338,12 +5338,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>osm_is_synthetic</t>
+          <t>poi_retail_food_count</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -5358,7 +5358,7 @@
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr">
         <is>
-          <t>True if osm used a synthetic fallback (raw source file missing).</t>
+          <t>Real OSM POI count: restaurants, cafes, fast food, shops.</t>
         </is>
       </c>
     </row>
@@ -5370,12 +5370,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>population_night</t>
+          <t>poi_office_count</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -5390,7 +5390,7 @@
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr">
         <is>
-          <t>Real WorldPop 2020 zonal-statistics residential population estimate for the cell.</t>
+          <t>Real OSM POI count: tagged office=*.</t>
         </is>
       </c>
     </row>
@@ -5402,12 +5402,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>population_density_per_km2</t>
+          <t>poi_recreation_count</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -5422,7 +5422,7 @@
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr">
         <is>
-          <t>population_night / real cell area (km^2, projected CRS).</t>
+          <t>Real OSM POI count: leisure=* or tourism=*.</t>
         </is>
       </c>
     </row>
@@ -5434,7 +5434,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>population_day</t>
+          <t>road_length_m</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -5454,7 +5454,7 @@
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Modelled daytime population (residential population reweighted by real OSM office/retail density) — explicitly an assumption, not a raster.</t>
+          <t>Real road length (m) per cell via polygon overlay in a projected CRS (not a heuristic).</t>
         </is>
       </c>
     </row>
@@ -5466,12 +5466,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>population_is_synthetic</t>
+          <t>road_density_km_per_km2</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -5486,7 +5486,7 @@
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr">
         <is>
-          <t>True if population used a synthetic fallback (raw source file missing).</t>
+          <t>road_length_m / 1000 / real cell area (km^2).</t>
         </is>
       </c>
     </row>
@@ -5498,16 +5498,16 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>ookla_dl_mbps</t>
+          <t>intersection_count</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>57.78</v>
+        <v>100</v>
       </c>
       <c r="E159" t="b">
         <v>1</v>
@@ -5518,7 +5518,7 @@
       <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr">
         <is>
-          <t>REAL Ookla tests-weighted mean download speed (Mbps) for the cell, static/quarterly. NaN where no tile coverage exists (not imputed).</t>
+          <t>Real OSM road-network node count per cell.</t>
         </is>
       </c>
     </row>
@@ -5530,7 +5530,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>ookla_rtt_ms</t>
+          <t>intersection_density_per_km2</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -5539,7 +5539,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>57.78</v>
+        <v>100</v>
       </c>
       <c r="E160" t="b">
         <v>1</v>
@@ -5550,7 +5550,7 @@
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="inlineStr">
         <is>
-          <t>REAL Ookla tests-weighted mean latency (ms) for the cell, static/quarterly. NaN where no tile coverage exists.</t>
+          <t>intersection_count / real cell area (km^2).</t>
         </is>
       </c>
     </row>
@@ -5562,7 +5562,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>ookla_tests</t>
+          <t>dist_to_nearest_transit_m</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -5571,7 +5571,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>57.78</v>
+        <v>100</v>
       </c>
       <c r="E161" t="b">
         <v>1</v>
@@ -5582,7 +5582,7 @@
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="inlineStr">
         <is>
-          <t>REAL summed Ookla test count backing ookla_dl_mbps/ookla_rtt_ms for the cell.</t>
+          <t>Real geometric nearest-neighbor distance to the nearest OSM transit/rail POI (sjoin_nearest, projected CRS).</t>
         </is>
       </c>
     </row>
@@ -5594,12 +5594,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>has_real_ookla_label</t>
+          <t>poi_transport_stop_count</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -5614,7 +5614,7 @@
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="inlineStr">
         <is>
-          <t>True if ookla_dl_mbps is non-null — i.e. this row has a REAL label usable for training in cell_static_qoe_baseline.parquet.</t>
+          <t>Real OSM POI count of public-transport/rail stops joined into the cell.</t>
         </is>
       </c>
     </row>
@@ -5626,16 +5626,16 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>qoe_risk_label</t>
+          <t>osm_is_synthetic</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>57.78</v>
+        <v>100</v>
       </c>
       <c r="E163" t="b">
         <v>1</v>
@@ -5646,147 +5646,147 @@
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="inlineStr">
         <is>
-          <t>high_risk/moderate_risk/low_risk from REAL ookla_dl_mbps thresholds. None where has_real_ookla_label is False (deliberately not guessed).</t>
+          <t>True if osm used a synthetic fallback (raw source file missing).</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>qoe_targets</t>
+          <t>cell_static_qoe_baseline</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>row_id</t>
+          <t>population_night</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D164" t="n">
         <v>100</v>
       </c>
       <c r="E164" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F164" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Surrogate unique row identifier (h3_index + timestamp composite, as int).</t>
+          <t>Real WorldPop 2020 zonal-statistics residential population estimate for the cell.</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>qoe_targets</t>
+          <t>cell_static_qoe_baseline</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>h3_index</t>
+          <t>population_density_per_km2</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D165" t="n">
         <v>100</v>
       </c>
       <c r="E165" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F165" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Uber H3 res-8 cell identifier (join key).</t>
+          <t>population_night / real cell area (km^2, projected CRS).</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>qoe_targets</t>
+          <t>cell_static_qoe_baseline</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>population_day</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>datetime64[us]</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D166" t="n">
         <v>100</v>
       </c>
       <c r="E166" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F166" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Hourly timestamp (UTC-naive, local Klang Valley convention).</t>
+          <t>Modelled daytime population (residential population reweighted by real OSM office/retail density) — explicitly an assumption, not a raster.</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>qoe_targets</t>
+          <t>cell_static_qoe_baseline</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>target_qoe_index</t>
+          <t>population_is_synthetic</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D167" t="n">
         <v>100</v>
       </c>
       <c r="E167" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F167" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Custom composite 0-100 QoE index (log-utility download/upload minus exponential latency/loss penalty). NOT a validated ITU-T G.107 MOS — see qoe_target.py docstring.</t>
+          <t>True if population used a synthetic fallback (raw source file missing).</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>qoe_targets</t>
+          <t>cell_static_qoe_baseline</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>target_service_quality_1to5</t>
+          <t>ookla_dl_mbps</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -5795,146 +5795,146 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>100</v>
+        <v>57.78</v>
       </c>
       <c r="E168" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F168" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1-5 linear rescaling of target_qoe_index. NOT a validated MOS/ACR score.</t>
+          <t>REAL Ookla tests-weighted mean download speed (Mbps) for the cell, static/quarterly. NaN where no tile coverage exists (not imputed).</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>qoe_targets</t>
+          <t>cell_static_qoe_baseline</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>target_is_degraded</t>
+          <t>ookla_rtt_ms</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>100</v>
+        <v>57.78</v>
       </c>
       <c r="E169" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F169" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Binary SAME-HOUR degradation flag, derived from target_degradation_class &gt;= 1 (single shared threshold source — config.QOE_THRESHOLDS — so this can no longer disagree with target_degradation_class).</t>
+          <t>REAL Ookla tests-weighted mean latency (ms) for the cell, static/quarterly. NaN where no tile coverage exists.</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>qoe_targets</t>
+          <t>cell_static_qoe_baseline</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>target_degradation_class</t>
+          <t>ookla_tests</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>100</v>
+        <v>57.78</v>
       </c>
       <c r="E170" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F170" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="inlineStr">
         <is>
-          <t>0=normal, 1=degraded, 2=severe. Same threshold source as target_is_degraded.</t>
+          <t>REAL summed Ookla test count backing ookla_dl_mbps/ookla_rtt_ms for the cell.</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>qoe_targets</t>
+          <t>cell_static_qoe_baseline</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>target_is_degraded_next_1h</t>
+          <t>has_real_ookla_label</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="E171" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F171" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="inlineStr">
         <is>
-          <t>RECOMMENDED PRIMARY ML TARGET. target_is_degraded shifted -1 per cell (groupby h3_index).shift(-1) — genuinely predicting the future, not classifying the present. NaN/0-valid for each cell's final row (no future observation exists).</t>
+          <t>True if ookla_dl_mbps is non-null — i.e. this row has a REAL label usable for training in cell_static_qoe_baseline.parquet.</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>qoe_targets</t>
+          <t>cell_static_qoe_baseline</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>target_degradation_class_next_1h</t>
+          <t>qoe_risk_label</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>99.40000000000001</v>
+        <v>57.78</v>
       </c>
       <c r="E172" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F172" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="inlineStr">
         <is>
-          <t>3-class version of the next-hour forecast target.</t>
+          <t>high_risk/moderate_risk/low_risk from REAL ookla_dl_mbps thresholds. None where has_real_ookla_label is False (deliberately not guessed).</t>
         </is>
       </c>
     </row>
@@ -5946,16 +5946,16 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>target_qoe_index_next_1h</t>
+          <t>row_id</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="E173" t="b">
         <v>0</v>
@@ -5966,7 +5966,7 @@
       <c r="G173" t="inlineStr"/>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Continuous version of the next-hour forecast target.</t>
+          <t>Surrogate unique row identifier (h3_index + timestamp composite, as int).</t>
         </is>
       </c>
     </row>
@@ -5978,12 +5978,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>target_next_1h_valid</t>
+          <t>h3_index</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -5998,7 +5998,7 @@
       <c r="G174" t="inlineStr"/>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1 if a real future observation existed to build the next-hour target from; 0 for each cell's final row. Drop rows where this is 0 before training — do not treat them as a 'not degraded' case.</t>
+          <t>Uber H3 res-8 cell identifier (join key).</t>
         </is>
       </c>
     </row>
@@ -6010,25 +6010,313 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>qoe_confidence_score</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>datetime64[us]</t>
         </is>
       </c>
       <c r="D175" t="n">
         <v>100</v>
       </c>
       <c r="E175" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F175" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G175" t="inlineStr"/>
       <c r="H175" t="inlineStr">
+        <is>
+          <t>Hourly timestamp (UTC-naive, local Klang Valley convention).</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>qoe_targets</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>target_qoe_index</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>float64</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>100</v>
+      </c>
+      <c r="E176" t="b">
+        <v>0</v>
+      </c>
+      <c r="F176" t="b">
+        <v>0</v>
+      </c>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Custom composite 0-100 QoE index (log-utility download/upload minus exponential latency/loss penalty). NOT a validated ITU-T G.107 MOS — see qoe_target.py docstring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>qoe_targets</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>target_service_quality_1to5</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>float64</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>100</v>
+      </c>
+      <c r="E177" t="b">
+        <v>0</v>
+      </c>
+      <c r="F177" t="b">
+        <v>0</v>
+      </c>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>1-5 linear rescaling of target_qoe_index. NOT a validated MOS/ACR score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>qoe_targets</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>target_is_degraded</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>int64</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>100</v>
+      </c>
+      <c r="E178" t="b">
+        <v>0</v>
+      </c>
+      <c r="F178" t="b">
+        <v>0</v>
+      </c>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Binary SAME-HOUR degradation flag, derived from target_degradation_class &gt;= 1 (single shared threshold source — config.QOE_THRESHOLDS — so this can no longer disagree with target_degradation_class).</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>qoe_targets</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>target_degradation_class</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>int64</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>100</v>
+      </c>
+      <c r="E179" t="b">
+        <v>0</v>
+      </c>
+      <c r="F179" t="b">
+        <v>0</v>
+      </c>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>0=normal, 1=degraded, 2=severe. Same threshold source as target_is_degraded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>qoe_targets</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>target_is_degraded_next_1h</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>float64</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="E180" t="b">
+        <v>0</v>
+      </c>
+      <c r="F180" t="b">
+        <v>0</v>
+      </c>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>RECOMMENDED PRIMARY ML TARGET. target_is_degraded shifted -1 per cell (groupby h3_index).shift(-1) — genuinely predicting the future, not classifying the present. NaN/0-valid for each cell's final row (no future observation exists).</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>qoe_targets</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>target_degradation_class_next_1h</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>float64</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="E181" t="b">
+        <v>0</v>
+      </c>
+      <c r="F181" t="b">
+        <v>0</v>
+      </c>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>3-class version of the next-hour forecast target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>qoe_targets</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>target_qoe_index_next_1h</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>float64</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="E182" t="b">
+        <v>0</v>
+      </c>
+      <c r="F182" t="b">
+        <v>0</v>
+      </c>
+      <c r="G182" t="inlineStr"/>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Continuous version of the next-hour forecast target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>qoe_targets</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>target_next_1h_valid</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>int64</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>100</v>
+      </c>
+      <c r="E183" t="b">
+        <v>0</v>
+      </c>
+      <c r="F183" t="b">
+        <v>0</v>
+      </c>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>1 if a real future observation existed to build the next-hour target from; 0 for each cell's final row. Drop rows where this is 0 before training — do not treat them as a 'not degraded' case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>qoe_targets</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>qoe_confidence_score</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>float64</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>100</v>
+      </c>
+      <c r="E184" t="b">
+        <v>1</v>
+      </c>
+      <c r="F184" t="b">
+        <v>1</v>
+      </c>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr">
         <is>
           <t>min(1.0, test_sample_count / 10) — higher sample count = more confidence in the cell-hour's QoE estimate.</t>
         </is>

</xml_diff>